<commit_message>
Product import: filters without images + link to compatible vehicles
- Filter-list column aliases (کد فنی، نام فیلتر، برند سازنده، نوع فیلتر)
  and optional «خودروهای سازگار» column; price no longer a required column
  and absent price/stock/carton columns don't overwrite existing values
- Exact-name vehicle matching; append-only «فیلتر» productLinks, report
  unmatched vehicles, filters without vehicles and in-file duplicates
- «Only new products» option leaves existing products untouched
- Brand-name placeholder image for brands without a logo

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/product-import-template.xlsx
+++ b/server/templates/product-import-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>کد محصول</t>
   </si>
@@ -74,6 +74,9 @@
     <t>نام فایل‌های گالری</t>
   </si>
   <si>
+    <t>خودروهای سازگار</t>
+  </si>
+  <si>
     <t>VAL-5W40-4L</t>
   </si>
   <si>
@@ -153,6 +156,9 @@
   </si>
   <si>
     <t>5. این فایل را همراه با پوشه عکس‌های محصولات، در بخش «ایمپورت گروهی محصولات» در پنل ادمین آپلود کنید.</t>
+  </si>
+  <si>
+    <t>6. عکس اختیاری است؛ محصول بدون عکس لوگوی برندش را نشان می‌دهد. ستون «خودروهای سازگار»: نام دقیق خودروها همان‌طور که در سایت ثبت شده‌اند، با کاما جدا (مثلاً: پژو 206 تیپ 2، سمند LX). محصول به تب فیلتر همان خودروها اضافه می‌شود و خودروهای پیدانشده در نتیجه‌ی ایمپورت گزارش می‌شوند.</t>
   </si>
 </sst>
 </file>
@@ -556,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="11" width="18" customWidth="1"/>
@@ -564,9 +570,10 @@
     <col min="18" max="18" width="20" customWidth="1"/>
     <col min="19" max="19" width="21" customWidth="1"/>
     <col min="20" max="20" width="22" customWidth="1"/>
+    <col min="21" max="21" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -627,67 +634,70 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -698,7 +708,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -706,37 +716,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>